<commit_message>
Added IIR, updated FIR interactive and dsp gen
</commit_message>
<xml_diff>
--- a/modules/fir_filter/filter spec calc.xlsx
+++ b/modules/fir_filter/filter spec calc.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\robot\OneDrive\Documents\VHDL\modules\fir_filter\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{360D5F3C-9975-4948-9FD4-FDF6C6C67856}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FAC946-BA47-422E-8831-7BA30402ADDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{AA2E42B5-DA60-480B-9FF6-CAACAEF237FF}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AA2E42B5-DA60-480B-9FF6-CAACAEF237FF}"/>
   </bookViews>
   <sheets>
     <sheet name="HPFLPF" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="109" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="128" uniqueCount="74">
   <si>
     <t>Fs</t>
   </si>
@@ -156,12 +156,6 @@
     <t>m!= 0</t>
   </si>
   <si>
-    <t>Index</t>
-  </si>
-  <si>
-    <t>m</t>
-  </si>
-  <si>
     <t>Lower Stop band</t>
   </si>
   <si>
@@ -186,16 +180,79 @@
     <t>fp2</t>
   </si>
   <si>
-    <t>Stop band edge</t>
-  </si>
-  <si>
-    <t>fl</t>
-  </si>
-  <si>
-    <t>Pass band edge</t>
-  </si>
-  <si>
-    <t>fh</t>
+    <t>Normalized lower stop band</t>
+  </si>
+  <si>
+    <t>fs1n</t>
+  </si>
+  <si>
+    <t>Normalized upper stop band</t>
+  </si>
+  <si>
+    <t>fs2n</t>
+  </si>
+  <si>
+    <t>Normalized lower pass band</t>
+  </si>
+  <si>
+    <t>fp1n</t>
+  </si>
+  <si>
+    <t>Normalized upper pass band</t>
+  </si>
+  <si>
+    <t>fp2n</t>
+  </si>
+  <si>
+    <t>Transition lower band</t>
+  </si>
+  <si>
+    <t>del f1</t>
+  </si>
+  <si>
+    <t>Transition upper band</t>
+  </si>
+  <si>
+    <t>del f2</t>
+  </si>
+  <si>
+    <t>Lowe cut off</t>
+  </si>
+  <si>
+    <t>fcl</t>
+  </si>
+  <si>
+    <t>Higher cut off</t>
+  </si>
+  <si>
+    <t>fch</t>
+  </si>
+  <si>
+    <t>normalized lower cut off</t>
+  </si>
+  <si>
+    <t>fln</t>
+  </si>
+  <si>
+    <t>Normalized higher cut off</t>
+  </si>
+  <si>
+    <t>fhn</t>
+  </si>
+  <si>
+    <t>m!=0</t>
+  </si>
+  <si>
+    <t>BPF</t>
+  </si>
+  <si>
+    <t>BSF</t>
+  </si>
+  <si>
+    <t>Denotion</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
 </sst>
 </file>
@@ -910,16 +967,21 @@
   <dimension ref="C3:M20"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="12.109375" style="5" customWidth="1"/>
+    <col min="3" max="3" width="19.88671875" style="5" customWidth="1"/>
     <col min="5" max="5" width="10" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="13" style="6" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="D3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3"/>
+      <c r="D3" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>73</v>
+      </c>
       <c r="F3" s="2" t="s">
         <v>22</v>
       </c>
@@ -1170,12 +1232,7 @@
       </c>
     </row>
     <row r="20" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C20" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>42</v>
-      </c>
+      <c r="D20" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1184,30 +1241,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F8E5DF94-F274-4F54-A22B-95F065739524}">
-  <dimension ref="C2:J23"/>
+  <dimension ref="C2:K27"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="19.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C2" s="12"/>
-      <c r="D2" s="12"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="12"/>
-    </row>
-    <row r="3" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="2" spans="3:11" x14ac:dyDescent="0.3">
+      <c r="C2" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>73</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C3" s="5"/>
-      <c r="D3" s="5" t="s">
-        <v>9</v>
-      </c>
       <c r="E3" s="12"/>
-      <c r="F3" s="5" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" spans="3:10" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="3:11" x14ac:dyDescent="0.3">
       <c r="C4" s="5" t="s">
         <v>18</v>
       </c>
@@ -1221,12 +1280,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="5" spans="3:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="3:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C5" s="5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E5" s="12">
         <v>14</v>
@@ -1235,12 +1294,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="3:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="3:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C6" s="5" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E6" s="12">
         <v>20</v>
@@ -1249,12 +1308,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="7" spans="3:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="3:11" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C7" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>47</v>
-      </c>
-      <c r="D7" s="12" t="s">
-        <v>49</v>
       </c>
       <c r="E7" s="12">
         <v>10</v>
@@ -1263,12 +1322,12 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="3:10" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="3:11" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D8" s="12" t="s">
         <v>48</v>
-      </c>
-      <c r="D8" s="12" t="s">
-        <v>50</v>
       </c>
       <c r="E8" s="12">
         <v>24</v>
@@ -1277,7 +1336,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="3:10" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="3:11" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C9" s="5" t="s">
         <v>21</v>
       </c>
@@ -1291,69 +1350,89 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="3:10" s="9" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="3:11" s="9" customFormat="1" x14ac:dyDescent="0.3">
       <c r="C10" s="10"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
-      <c r="I10" s="11"/>
-    </row>
-    <row r="11" spans="3:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I10" s="11" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C11" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" s="3">
-        <f>(E5+E6)/2</f>
-        <v>17</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I11" s="1"/>
-      <c r="J11" s="1"/>
-    </row>
-    <row r="12" spans="3:10" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C12" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="3">
-        <f>(E8+E7)/2</f>
-        <v>17</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="I12" s="1"/>
-      <c r="J12" s="1"/>
-    </row>
-    <row r="13" spans="3:10" ht="18.600000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D13" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="E13" s="12">
+        <v>49</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="12">
         <f>E5/E4</f>
         <v>0.17499999999999999</v>
       </c>
+      <c r="F11" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" s="1"/>
+      <c r="J11" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>52</v>
+      </c>
+      <c r="E12" s="12">
+        <f>E6/E4</f>
+        <v>0.25</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="H12" s="1"/>
+      <c r="I12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="J12">
+        <f>2*(E22-E21)</f>
+        <v>0.25000000000000006</v>
+      </c>
+      <c r="K12">
+        <f>1-J12</f>
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="E13" s="12">
+        <f>E7/E4</f>
+        <v>0.125</v>
+      </c>
       <c r="F13" s="12" t="s">
         <v>26</v>
       </c>
       <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="3:10" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I13" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C14" s="5" t="s">
-        <v>12</v>
+        <v>55</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="E14" s="12">
         <f>E8/E4</f>
@@ -1364,133 +1443,195 @@
       </c>
       <c r="H14" s="1"/>
     </row>
-    <row r="15" spans="3:10" ht="20.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C15" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="D15" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="E15" s="12">
+        <f>E5-E7</f>
+        <v>4</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H15" s="1"/>
+    </row>
+    <row r="16" spans="3:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C16" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="E16" s="12">
+        <f>E8-E6</f>
+        <v>4</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="H16" s="1"/>
+    </row>
+    <row r="17" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C17" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D17" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="E15" s="12">
-        <f>3/48</f>
-        <v>6.25E-2</v>
-      </c>
-      <c r="F15" s="12" t="s">
+      <c r="E17" s="12">
+        <f>E16/E4</f>
+        <v>0.05</v>
+      </c>
+      <c r="F17" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="16" spans="3:10" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C16" s="5" t="s">
+    <row r="18" spans="3:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C18" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D18" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="E16" s="12">
-        <f>2*3.14*E15</f>
-        <v>0.39250000000000002</v>
-      </c>
-      <c r="F16" s="12" t="s">
+      <c r="E18" s="12">
+        <f>2*3.14*E17</f>
+        <v>0.31400000000000006</v>
+      </c>
+      <c r="F18" s="12" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="3:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C17" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>4</v>
-      </c>
-      <c r="E17" s="12">
-        <f>(E8+E5)/2</f>
-        <v>19</v>
-      </c>
-      <c r="F17" s="12" t="s">
+    <row r="19" spans="3:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C19" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="12">
+        <f>(E5+E7)/2</f>
+        <v>12</v>
+      </c>
+      <c r="F19" s="12" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="18" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="C18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="D18" s="12" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="12">
-        <f>E17/E4</f>
-        <v>0.23749999999999999</v>
-      </c>
-      <c r="F18" s="12" t="s">
+    <row r="20" spans="3:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C20" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="E20" s="12">
+        <f>(E8+E6)/2</f>
+        <v>22</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="21" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="C21" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="E21" s="12">
+        <f>E19/E4</f>
+        <v>0.15</v>
+      </c>
+      <c r="F21" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="19" spans="3:6" x14ac:dyDescent="0.3">
-      <c r="C19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="D19" s="12" t="s">
-        <v>8</v>
-      </c>
-      <c r="E19" s="12">
-        <f>(0.5842*POWER((E9-21),0.4))+(0.07886*(E9-21))</f>
-        <v>5.6047645895609897</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="20" spans="3:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C20" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="D20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E20" s="12">
-        <f>((E9-7.95)/(2.285*E16))+1</f>
-        <v>59.03565206483713</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="21" spans="3:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D21" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="E21" s="12">
-        <v>49</v>
-      </c>
-      <c r="F21" s="12"/>
-    </row>
-    <row r="22" spans="3:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="3:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="C22" s="5" t="s">
-        <v>30</v>
+        <v>67</v>
       </c>
       <c r="D22" s="12" t="s">
-        <v>31</v>
+        <v>68</v>
       </c>
       <c r="E22" s="12">
-        <f>(E21-1)/2</f>
-        <v>24</v>
-      </c>
-      <c r="F22" s="12"/>
+        <f>E20/E4</f>
+        <v>0.27500000000000002</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="23" spans="3:6" x14ac:dyDescent="0.3">
       <c r="C23" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E23" s="12">
+        <f>0.1102*(E9-8.7)</f>
+        <v>5.6532600000000004</v>
+      </c>
+      <c r="F23" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="24" spans="3:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" s="12">
+        <f>((E9-7.95)/(2.285*E18))+1</f>
+        <v>73.5445650810464</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="25" spans="3:6" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C25" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="E25" s="12">
+        <v>75</v>
+      </c>
+      <c r="F25" s="12"/>
+    </row>
+    <row r="26" spans="3:6" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C26" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="E26" s="12">
+        <f>(E25-1)/2</f>
+        <v>37</v>
+      </c>
+      <c r="F26" s="12"/>
+    </row>
+    <row r="27" spans="3:6" x14ac:dyDescent="0.3">
+      <c r="C27" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="D23" s="12" t="s">
+      <c r="D27" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="E23" s="12">
-        <f>E22/(E4*10^6)</f>
-        <v>2.9999999999999999E-7</v>
-      </c>
-      <c r="F23" s="12" t="s">
+      <c r="E27" s="12">
+        <f>E26/(E4*10^6)</f>
+        <v>4.6250000000000002E-7</v>
+      </c>
+      <c r="F27" s="12" t="s">
         <v>35</v>
       </c>
     </row>

</xml_diff>